<commit_message>
fix(pedido): se quita el check 'Cant. fija' del formulario, del modelo y de las plantillas — la cantidad del pedido es el total del servicio
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/public/plantillas/pedido-fcr-sarta-limpieza-4426.xlsx
+++ b/public/plantillas/pedido-fcr-sarta-limpieza-4426.xlsx
@@ -427,7 +427,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G8"/>
+  <dimension ref="A1:F8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -436,13 +436,12 @@
     <col width="70" customWidth="1" min="4" max="4"/>
     <col width="12" customWidth="1" min="5" max="5"/>
     <col width="20" customWidth="1" min="6" max="6"/>
-    <col width="15" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>Plantilla de pedido de ejemplo — formato AS2 Pedido Cliente (columna G opcional: Cantidad fija)</t>
+          <t>Plantilla de pedido de ejemplo — formato AS2 Pedido Cliente</t>
         </is>
       </c>
     </row>
@@ -508,11 +507,6 @@
           <t>Porcentaje Descuento</t>
         </is>
       </c>
-      <c r="G4" s="2" t="inlineStr">
-        <is>
-          <t>Cantidad fija</t>
-        </is>
-      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -539,11 +533,6 @@
       <c r="F5" t="n">
         <v>0</v>
       </c>
-      <c r="G5" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -570,11 +559,6 @@
       <c r="F6" t="n">
         <v>0</v>
       </c>
-      <c r="G6" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -601,11 +585,6 @@
       <c r="F7" t="n">
         <v>0</v>
       </c>
-      <c r="G7" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -631,11 +610,6 @@
       </c>
       <c r="F8" t="n">
         <v>0</v>
-      </c>
-      <c r="G8" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>